<commit_message>
The recording comes off yes
</commit_message>
<xml_diff>
--- a/lexicon/lexicon.xlsx
+++ b/lexicon/lexicon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Github\upta\khallam\lexicon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C204FBB7-FCD1-4F41-9176-36ABD5BE0EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E772B7-8EE2-4270-B62F-3363D817E461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="325">
   <si>
     <t>id (filled in for you)</t>
   </si>
@@ -935,9 +935,6 @@
   </si>
   <si>
     <t>m̓</t>
-  </si>
-  <si>
-    <t>yes.mp3</t>
   </si>
   <si>
     <t>you</t>
@@ -1420,7 +1417,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
@@ -1476,7 +1473,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>16</v>
@@ -1686,7 +1683,7 @@
         <v>63</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>64</v>
@@ -2607,7 +2604,7 @@
         <v>270</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>271</v>
@@ -2749,78 +2746,75 @@
       <c r="C97" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="D97" s="2" t="s">
-        <v>305</v>
-      </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B98" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="C98" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B99" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="C99" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="D99" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B100" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="B100" s="2" t="s">
-        <v>314</v>
-      </c>
       <c r="C100" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D100" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B101" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="C101" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="D101" s="2" t="s">
         <v>317</v>
-      </c>
-      <c r="D101" s="2" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
+        <v>319</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D102" s="2" t="s">
         <v>320</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add the alphabet sounds and point the guide at them
</commit_message>
<xml_diff>
--- a/lexicon/lexicon.xlsx
+++ b/lexicon/lexicon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Github\upta\khallam\lexicon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E009B29-C591-4556-BEA8-C9725B6F026F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D957AC6-ABDE-44E5-AD7E-A934F55E74BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10695" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lexicon" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="467">
   <si>
     <t>id (filled in for you)</t>
   </si>
@@ -1238,6 +1238,189 @@
   </si>
   <si>
     <t>pronouns</t>
+  </si>
+  <si>
+    <t>run-away</t>
+  </si>
+  <si>
+    <t>get-dressed</t>
+  </si>
+  <si>
+    <t>help-it-him-her-them</t>
+  </si>
+  <si>
+    <t>look-at-it</t>
+  </si>
+  <si>
+    <t>wake-it</t>
+  </si>
+  <si>
+    <t>dry-it</t>
+  </si>
+  <si>
+    <t>hold-it</t>
+  </si>
+  <si>
+    <t>hit-it</t>
+  </si>
+  <si>
+    <t>lift-it</t>
+  </si>
+  <si>
+    <t>choose-it</t>
+  </si>
+  <si>
+    <t>break-it-long-object</t>
+  </si>
+  <si>
+    <t>take-it</t>
+  </si>
+  <si>
+    <t>young-man</t>
+  </si>
+  <si>
+    <t>old-animate</t>
+  </si>
+  <si>
+    <t>old-worn-out-thing</t>
+  </si>
+  <si>
+    <t>i-intransitive</t>
+  </si>
+  <si>
+    <t>we-intransitive</t>
+  </si>
+  <si>
+    <t>you-intransitive</t>
+  </si>
+  <si>
+    <t>you-all-you-folks-intransitive</t>
+  </si>
+  <si>
+    <t>he-she-it-they-transitive-suffix</t>
+  </si>
+  <si>
+    <t>the-that-specific-article</t>
+  </si>
+  <si>
+    <t>glottal stop</t>
+  </si>
+  <si>
+    <t>schwa</t>
+  </si>
+  <si>
+    <t>uvular fricative</t>
+  </si>
+  <si>
+    <t>rounded velar fricative</t>
+  </si>
+  <si>
+    <t>voiceless lateral</t>
+  </si>
+  <si>
+    <t>ch sound</t>
+  </si>
+  <si>
+    <t>ejective lateral</t>
+  </si>
+  <si>
+    <t>uvular k</t>
+  </si>
+  <si>
+    <t>rounded uvular k</t>
+  </si>
+  <si>
+    <t>ejective p</t>
+  </si>
+  <si>
+    <t>ejective t</t>
+  </si>
+  <si>
+    <t>ejective k</t>
+  </si>
+  <si>
+    <t>stressed a</t>
+  </si>
+  <si>
+    <t>stressed e</t>
+  </si>
+  <si>
+    <t>stressed i</t>
+  </si>
+  <si>
+    <t>stressed schwa</t>
+  </si>
+  <si>
+    <t>stressed u</t>
+  </si>
+  <si>
+    <t>glottalized n</t>
+  </si>
+  <si>
+    <t>glottalized y</t>
+  </si>
+  <si>
+    <t>sh sound</t>
+  </si>
+  <si>
+    <t>ʔ</t>
+  </si>
+  <si>
+    <t>ə</t>
+  </si>
+  <si>
+    <t>x̣</t>
+  </si>
+  <si>
+    <t>xʷ</t>
+  </si>
+  <si>
+    <t>ɬ</t>
+  </si>
+  <si>
+    <t>č</t>
+  </si>
+  <si>
+    <t>ƛ̓</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>qʷ</t>
+  </si>
+  <si>
+    <t>p̓</t>
+  </si>
+  <si>
+    <t>t̓</t>
+  </si>
+  <si>
+    <t>k̓</t>
+  </si>
+  <si>
+    <t>á</t>
+  </si>
+  <si>
+    <t>é</t>
+  </si>
+  <si>
+    <t>í</t>
+  </si>
+  <si>
+    <t>ə́</t>
+  </si>
+  <si>
+    <t>ú</t>
+  </si>
+  <si>
+    <t>n̓</t>
+  </si>
+  <si>
+    <t>y̓</t>
+  </si>
+  <si>
+    <t>š</t>
   </si>
 </sst>
 </file>
@@ -1645,8 +1828,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E139"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E159"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" style="3" customWidth="1"/>
     <col min="2" max="2" width="22" style="2" customWidth="1"/>
@@ -1655,7 +1838,7 @@
     <col min="5" max="5" width="24" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1672,7 +1855,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">afraid</t>
@@ -1688,7 +1871,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">all</t>
@@ -1704,7 +1887,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">basket</t>
@@ -1720,7 +1903,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">big</t>
@@ -1739,7 +1922,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">bird</t>
@@ -1755,7 +1938,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">black</t>
@@ -1774,7 +1957,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">blackberry</t>
@@ -1790,7 +1973,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">bone-game</t>
@@ -1806,7 +1989,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">bread</t>
@@ -1822,7 +2005,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">canoe</t>
@@ -1841,7 +2024,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">cat</t>
@@ -1860,7 +2043,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">cedar-wood</t>
@@ -1876,7 +2059,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">chinook-salmon</t>
@@ -1892,7 +2075,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">coat</t>
@@ -1908,7 +2091,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">comb</t>
@@ -1924,7 +2107,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">continue</t>
@@ -1940,7 +2123,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">cow</t>
@@ -1956,7 +2139,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">crab</t>
@@ -1972,7 +2155,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">cry</t>
@@ -1991,7 +2174,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">cut-it</t>
@@ -2010,7 +2193,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">day</t>
@@ -2026,7 +2209,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">deer</t>
@@ -2045,7 +2228,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">dirt</t>
@@ -2061,7 +2244,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">disappear</t>
@@ -2077,7 +2260,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">dog</t>
@@ -2096,7 +2279,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">duck</t>
@@ -2112,7 +2295,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">ear</t>
@@ -2128,7 +2311,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">eat</t>
@@ -2144,7 +2327,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">elwha</t>
@@ -2160,7 +2343,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">enter</t>
@@ -2176,7 +2359,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">evening</t>
@@ -2192,7 +2375,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">finish</t>
@@ -2208,7 +2391,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">five</t>
@@ -2224,7 +2407,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">flip</t>
@@ -2240,7 +2423,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">flounder</t>
@@ -2256,7 +2439,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">foot</t>
@@ -2272,7 +2455,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">four</t>
@@ -2288,7 +2471,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">go</t>
@@ -2307,7 +2490,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">go-home</t>
@@ -2323,7 +2506,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">go-with</t>
@@ -2339,7 +2522,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">good</t>
@@ -2358,7 +2541,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">goodbye</t>
@@ -2374,7 +2557,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hand</t>
@@ -2390,7 +2573,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hat</t>
@@ -2406,7 +2589,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">heart</t>
@@ -2422,7 +2605,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">house</t>
@@ -2441,7 +2624,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">how-many</t>
@@ -2457,7 +2640,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hungry</t>
@@ -2473,7 +2656,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">important-person</t>
@@ -2489,7 +2672,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">jellyfish</t>
@@ -2505,7 +2688,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">key</t>
@@ -2521,7 +2704,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">know-it</t>
@@ -2540,7 +2723,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">laugh</t>
@@ -2556,7 +2739,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">like</t>
@@ -2572,7 +2755,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">long</t>
@@ -2588,7 +2771,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">man</t>
@@ -2604,7 +2787,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">mother</t>
@@ -2623,7 +2806,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">mouth</t>
@@ -2639,7 +2822,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">much</t>
@@ -2658,7 +2841,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">my-child</t>
@@ -2674,7 +2857,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">new</t>
@@ -2693,7 +2876,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">one</t>
@@ -2709,7 +2892,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">outside</t>
@@ -2725,7 +2908,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">play</t>
@@ -2741,7 +2924,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">potato</t>
@@ -2757,7 +2940,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">raccoon</t>
@@ -2773,7 +2956,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">rat</t>
@@ -2789,7 +2972,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">road-door</t>
@@ -2808,7 +2991,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sack</t>
@@ -2821,7 +3004,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">scratch</t>
@@ -2837,7 +3020,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sheep</t>
@@ -2853,7 +3036,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sit-down</t>
@@ -2869,7 +3052,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">six</t>
@@ -2885,7 +3068,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">skin-hide</t>
@@ -2901,7 +3084,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sleep</t>
@@ -2920,7 +3103,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">small</t>
@@ -2939,7 +3122,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sneezing</t>
@@ -2955,7 +3138,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">stick</t>
@@ -2974,7 +3157,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">strong</t>
@@ -2993,7 +3176,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">talking</t>
@@ -3009,7 +3192,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">ten</t>
@@ -3025,7 +3208,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">three</t>
@@ -3041,7 +3224,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">tide</t>
@@ -3057,7 +3240,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">tongue</t>
@@ -3073,7 +3256,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">tooth</t>
@@ -3089,7 +3272,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">trying-it</t>
@@ -3102,7 +3285,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">uncle-aunt</t>
@@ -3121,7 +3304,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">walk</t>
@@ -3140,7 +3323,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">water</t>
@@ -3159,7 +3342,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">what</t>
@@ -3175,7 +3358,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">whistle</t>
@@ -3191,7 +3374,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">white</t>
@@ -3210,7 +3393,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">white-person</t>
@@ -3226,7 +3409,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">who</t>
@@ -3242,7 +3425,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">wishing</t>
@@ -3258,7 +3441,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
@@ -3271,7 +3454,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">you</t>
@@ -3287,7 +3470,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">young-woman</t>
@@ -3306,7 +3489,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">young-woman-2</t>
@@ -3322,7 +3505,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">your-mother</t>
@@ -3338,7 +3521,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">two</t>
@@ -3354,7 +3537,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">run</t>
@@ -3370,7 +3553,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">dive</t>
@@ -3386,7 +3569,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">fly</t>
@@ -3402,7 +3585,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">run-away</t>
@@ -3418,7 +3601,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">jump</t>
@@ -3434,7 +3617,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">grow</t>
@@ -3450,7 +3633,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">get-dressed</t>
@@ -3466,7 +3649,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">help-it-him-her-them</t>
@@ -3482,7 +3665,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">look-at-it</t>
@@ -3498,7 +3681,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">wake-it</t>
@@ -3514,7 +3697,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="113" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">dry-it</t>
@@ -3530,7 +3713,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="114" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hold-it</t>
@@ -3546,7 +3729,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="115" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hit-it</t>
@@ -3562,7 +3745,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="116" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">lift-it</t>
@@ -3578,7 +3761,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="117" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">choose-it</t>
@@ -3594,7 +3777,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="118" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">break-it-long-object</t>
@@ -3610,7 +3793,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="119" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">take-it</t>
@@ -3626,7 +3809,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="120" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">father</t>
@@ -3642,7 +3825,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="121" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">money</t>
@@ -3658,7 +3841,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="122" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">young-man</t>
@@ -3674,7 +3857,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="123" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">friend</t>
@@ -3690,7 +3873,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="124" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">word</t>
@@ -3706,7 +3889,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="125" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">bad</t>
@@ -3722,7 +3905,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="126" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">old-animate</t>
@@ -3738,7 +3921,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="127" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">old-worn-out-thing</t>
@@ -3754,7 +3937,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="128" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">fast</t>
@@ -3770,7 +3953,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="129" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">i-intransitive</t>
@@ -3786,7 +3969,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="130" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">we-intransitive</t>
@@ -3802,7 +3985,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="131" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">you-intransitive</t>
@@ -3818,7 +4001,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="132" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">you-all-you-folks-intransitive</t>
@@ -3834,7 +4017,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="133" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">he-she-it-they-transitive-suffix</t>
@@ -3850,7 +4033,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="134" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">the-that-specific-article</t>
@@ -3866,7 +4049,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="135" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">your</t>
@@ -3879,7 +4062,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="136" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">work</t>
@@ -3892,7 +4075,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="137" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">salt</t>
@@ -3905,7 +4088,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="138" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">raven</t>
@@ -3918,7 +4101,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="139" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">grandparent</t>
@@ -3929,6 +4112,266 @@
       </c>
       <c r="C139" s="2" t="s">
         <v>404</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">glottal-stop</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">schwa</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uvular-fricative</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rounded-velar-fricative</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">voiceless-lateral</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ch-sound</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ejective-lateral</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uvular-k</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rounded-uvular-k</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ejective-p</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ejective-t</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ejective-k</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="152" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stressed-a</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="153" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stressed-e</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stressed-i</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stressed-schwa</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stressed-u</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">glottalized-n</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="158" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">glottalized-y</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="159" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sh-sound</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>